<commit_message>
Excel Topics Covered:Pivot table and VLOOKUP
</commit_message>
<xml_diff>
--- a/excel_01_basics_functions.xlsx
+++ b/excel_01_basics_functions.xlsx
@@ -8,17 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a2438f9ef33e3037/Desktop/Data Analytics Preparation/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{2142660C-5A72-4853-8FA7-40FFBD1099CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81C331E2-0805-46B2-B57A-25713B6C2938}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="8_{2142660C-5A72-4853-8FA7-40FFBD1099CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97E72B31-2FE1-42DF-A1EE-F149757466BE}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E40E206A-CD2F-44D4-8383-96E00DEA2B61}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{E40E206A-CD2F-44D4-8383-96E00DEA2B61}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId2"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Sheet1!$A$1:$F$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="0" r:id="rId5"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="28">
   <si>
     <t>Order ID</t>
   </si>
@@ -100,6 +106,27 @@
   </si>
   <si>
     <t>Performance</t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Sum of Sales</t>
+  </si>
+  <si>
+    <t>Sum of Profit</t>
+  </si>
+  <si>
+    <t>Sum of Quantity</t>
+  </si>
+  <si>
+    <t>Column Labels</t>
+  </si>
+  <si>
+    <t>Tax Rate</t>
   </si>
 </sst>
 </file>
@@ -201,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -238,6 +265,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -253,6 +284,1522 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[excel_01_basics_functions.xlsx]Sheet2!PivotTable1</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Sales and Profit by Category</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-IN"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-IN"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$B$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of Sales</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$4:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Furniture</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Office Supplies</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Technology</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$4:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>17400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4050</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>37500</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-BB2C-4632-9D56-2E7C471E7FF9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$C$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of Profit</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$4:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Furniture</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Office Supplies</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Technology</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$C$4:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>3480</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>810</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9375</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-BB2C-4632-9D56-2E7C471E7FF9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="182"/>
+        <c:axId val="441671839"/>
+        <c:axId val="441700159"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="441671839"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="441700159"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="441700159"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="441671839"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>99060</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>403860</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52179B56-AF82-354D-7EE0-4D61B642A242}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Manasa" refreshedDate="46171.870899189817" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="12" xr:uid="{78E21158-7A13-467B-9FE7-8E0892D5F3A3}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:G13" sheet="Sheet1"/>
+  </cacheSource>
+  <cacheFields count="7">
+    <cacheField name="Order ID" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1001" maxValue="1012"/>
+    </cacheField>
+    <cacheField name="Category" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Furniture"/>
+        <s v="Technology"/>
+        <s v="Office Supplies"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Region" numFmtId="0">
+      <sharedItems count="4">
+        <s v="South"/>
+        <s v="West"/>
+        <s v="East"/>
+        <s v="North"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Sales" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="800" maxValue="12000"/>
+    </cacheField>
+    <cacheField name="Profit" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="160" maxValue="3000"/>
+    </cacheField>
+    <cacheField name="Quantity" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="6"/>
+    </cacheField>
+    <cacheField name="Performance" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="12">
+  <r>
+    <n v="1001"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="4500"/>
+    <n v="900"/>
+    <n v="3"/>
+    <s v="Low"/>
+  </r>
+  <r>
+    <n v="1002"/>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="8200"/>
+    <n v="2050"/>
+    <n v="2"/>
+    <s v="High"/>
+  </r>
+  <r>
+    <n v="1003"/>
+    <x v="2"/>
+    <x v="2"/>
+    <n v="1200"/>
+    <n v="240"/>
+    <n v="5"/>
+    <s v="Low"/>
+  </r>
+  <r>
+    <n v="1004"/>
+    <x v="0"/>
+    <x v="2"/>
+    <n v="3100"/>
+    <n v="620"/>
+    <n v="4"/>
+    <s v="Low"/>
+  </r>
+  <r>
+    <n v="1005"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="9500"/>
+    <n v="2375"/>
+    <n v="1"/>
+    <s v="High"/>
+  </r>
+  <r>
+    <n v="1006"/>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="800"/>
+    <n v="160"/>
+    <n v="6"/>
+    <s v="Low"/>
+  </r>
+  <r>
+    <n v="1007"/>
+    <x v="0"/>
+    <x v="1"/>
+    <n v="5600"/>
+    <n v="1120"/>
+    <n v="2"/>
+    <s v="High"/>
+  </r>
+  <r>
+    <n v="1008"/>
+    <x v="1"/>
+    <x v="2"/>
+    <n v="12000"/>
+    <n v="3000"/>
+    <n v="3"/>
+    <s v="High"/>
+  </r>
+  <r>
+    <n v="1009"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="950"/>
+    <n v="190"/>
+    <n v="4"/>
+    <s v="Low"/>
+  </r>
+  <r>
+    <n v="1010"/>
+    <x v="0"/>
+    <x v="3"/>
+    <n v="4200"/>
+    <n v="840"/>
+    <n v="5"/>
+    <s v="Low"/>
+  </r>
+  <r>
+    <n v="1011"/>
+    <x v="1"/>
+    <x v="3"/>
+    <n v="7800"/>
+    <n v="1950"/>
+    <n v="2"/>
+    <s v="High"/>
+  </r>
+  <r>
+    <n v="1012"/>
+    <x v="2"/>
+    <x v="3"/>
+    <n v="1100"/>
+    <n v="220"/>
+    <n v="3"/>
+    <s v="Low"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{49B33C11-E412-41AF-A3ED-6E672977989B}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="A3:C7" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="7">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Profit" fld="4" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA7384AF-D679-4CD7-8425-F679F323F79E}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="7">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Quantity" fld="5" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B6FC0A21-EBA0-453A-B817-349FA7D7F405}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:F8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="7">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -551,16 +2098,293 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3504E86C-49E1-4945-B212-5838C5EF21DB}">
+  <dimension ref="A3:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>17400</v>
+      </c>
+      <c r="C4">
+        <v>3480</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>4050</v>
+      </c>
+      <c r="C5">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>37500</v>
+      </c>
+      <c r="C6">
+        <v>9375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7">
+        <v>58950</v>
+      </c>
+      <c r="C7">
+        <v>13665</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C3049D-3A0E-474A-B83F-9E411026868B}">
+  <dimension ref="A3:C8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>16300</v>
+      </c>
+      <c r="C4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>13100</v>
+      </c>
+      <c r="C5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>14950</v>
+      </c>
+      <c r="C6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>14600</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8">
+        <v>58950</v>
+      </c>
+      <c r="C8">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23046505-D60C-47ED-AE29-4BEB518FAB00}">
+  <dimension ref="A3:F8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>3100</v>
+      </c>
+      <c r="C5">
+        <v>4200</v>
+      </c>
+      <c r="D5">
+        <v>4500</v>
+      </c>
+      <c r="E5">
+        <v>5600</v>
+      </c>
+      <c r="F5">
+        <v>17400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>1200</v>
+      </c>
+      <c r="C6">
+        <v>1100</v>
+      </c>
+      <c r="D6">
+        <v>950</v>
+      </c>
+      <c r="E6">
+        <v>800</v>
+      </c>
+      <c r="F6">
+        <v>4050</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>12000</v>
+      </c>
+      <c r="C7">
+        <v>7800</v>
+      </c>
+      <c r="D7">
+        <v>9500</v>
+      </c>
+      <c r="E7">
+        <v>8200</v>
+      </c>
+      <c r="F7">
+        <v>37500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8">
+        <v>16300</v>
+      </c>
+      <c r="C8">
+        <v>13100</v>
+      </c>
+      <c r="D8">
+        <v>14950</v>
+      </c>
+      <c r="E8">
+        <v>14600</v>
+      </c>
+      <c r="F8">
+        <v>58950</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F5DFD9-2BE5-40DD-A037-13E69B8EBBED}">
-  <dimension ref="A1:G344"/>
+  <dimension ref="A1:K344"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" customWidth="1"/>
     <col min="2" max="2" width="11.5546875" customWidth="1"/>
     <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -582,8 +2406,17 @@
       <c r="G1" s="13" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="13">
         <v>1001</v>
       </c>
@@ -603,11 +2436,21 @@
         <v>3</v>
       </c>
       <c r="G2" t="str">
-        <f>IF(D2&gt;5000,"High","Low")</f>
+        <f t="shared" ref="G2:G13" si="0">IF(D2&gt;5000,"High","Low")</f>
         <v>Low</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2">
+        <f>VLOOKUP(B2,$J$2:$K$4,2,FALSE)</f>
+        <v>0.12</v>
+      </c>
+      <c r="J2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="13">
         <v>1002</v>
       </c>
@@ -627,11 +2470,21 @@
         <v>2</v>
       </c>
       <c r="G3" t="str">
-        <f>IF(D3&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>High</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H3">
+        <f t="shared" ref="H3:H13" si="1">VLOOKUP(B3,$J$2:$K$4,2,FALSE)</f>
+        <v>0.18</v>
+      </c>
+      <c r="J3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K3">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="13">
         <v>1003</v>
       </c>
@@ -651,11 +2504,21 @@
         <v>5</v>
       </c>
       <c r="G4" t="str">
-        <f>IF(D4&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>Low</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+      <c r="J4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
         <v>1004</v>
       </c>
@@ -675,11 +2538,15 @@
         <v>4</v>
       </c>
       <c r="G5" t="str">
-        <f>IF(D5&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>Low</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5">
+        <f t="shared" si="1"/>
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="13">
         <v>1005</v>
       </c>
@@ -699,11 +2566,15 @@
         <v>1</v>
       </c>
       <c r="G6" t="str">
-        <f>IF(D6&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>High</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H6">
+        <f t="shared" si="1"/>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="13">
         <v>1006</v>
       </c>
@@ -723,11 +2594,15 @@
         <v>6</v>
       </c>
       <c r="G7" t="str">
-        <f>IF(D7&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>Low</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
         <v>1007</v>
       </c>
@@ -747,11 +2622,15 @@
         <v>2</v>
       </c>
       <c r="G8" t="str">
-        <f>IF(D8&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>High</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8">
+        <f t="shared" si="1"/>
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
         <v>1008</v>
       </c>
@@ -771,11 +2650,15 @@
         <v>3</v>
       </c>
       <c r="G9" t="str">
-        <f>IF(D9&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>High</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H9">
+        <f t="shared" si="1"/>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="13">
         <v>1009</v>
       </c>
@@ -795,11 +2678,15 @@
         <v>4</v>
       </c>
       <c r="G10" t="str">
-        <f>IF(D10&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>Low</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H10">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
         <v>1010</v>
       </c>
@@ -819,11 +2706,15 @@
         <v>5</v>
       </c>
       <c r="G11" t="str">
-        <f>IF(D11&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>Low</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H11">
+        <f t="shared" si="1"/>
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
         <v>1011</v>
       </c>
@@ -843,11 +2734,15 @@
         <v>2</v>
       </c>
       <c r="G12" t="str">
-        <f>IF(D12&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>High</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H12">
+        <f t="shared" si="1"/>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="13">
         <v>1012</v>
       </c>
@@ -867,16 +2762,20 @@
         <v>3</v>
       </c>
       <c r="G13" t="str">
-        <f>IF(D13&gt;5000,"High","Low")</f>
+        <f t="shared" si="0"/>
         <v>Low</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H13">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="13" t="s">
         <v>15</v>

</xml_diff>